<commit_message>
Décisions : 15 correspondances confirmées pour octobre 2026 (v4), mémoire créée
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KigtzRHCW12SnFTssRcRrW
</commit_message>
<xml_diff>
--- a/outputs/import-mensuel-finance/runs/Database XBH Octobre 2026 v4.xlsx
+++ b/outputs/import-mensuel-finance/runs/Database XBH Octobre 2026 v4.xlsx
@@ -16935,9 +16935,14 @@
       <c r="D2" t="n">
         <v>0.5</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -16966,9 +16971,14 @@
       <c r="D3" t="n">
         <v>0.5</v>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -16997,9 +17007,14 @@
       <c r="D4" t="n">
         <v>0.5</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -17028,9 +17043,14 @@
       <c r="D5" t="n">
         <v>1</v>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -17059,9 +17079,14 @@
       <c r="D6" t="n">
         <v>1</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -17090,9 +17115,14 @@
       <c r="D7" t="n">
         <v>0.5</v>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -17121,9 +17151,14 @@
       <c r="D8" t="n">
         <v>1</v>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -17152,9 +17187,14 @@
       <c r="D9" t="n">
         <v>0.5</v>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -17183,9 +17223,14 @@
       <c r="D10" t="n">
         <v>0.5</v>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -17214,9 +17259,14 @@
       <c r="D11" t="n">
         <v>0.5</v>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -17245,9 +17295,14 @@
       <c r="D12" t="n">
         <v>1</v>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -17276,9 +17331,14 @@
       <c r="D13" t="n">
         <v>1</v>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -17307,9 +17367,14 @@
       <c r="D14" t="n">
         <v>0.5</v>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G14" t="n">
@@ -17338,9 +17403,14 @@
       <c r="D15" t="n">
         <v>0.5</v>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -17369,9 +17439,14 @@
       <c r="D16" t="n">
         <v>0.5</v>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G16" t="n">
@@ -17392,7 +17467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17456,7 +17531,7 @@
         <v>49730715.52</v>
       </c>
       <c r="F2" t="n">
-        <v>62990146.13</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -17486,7 +17561,7 @@
         <v>47409793.37</v>
       </c>
       <c r="F3" t="n">
-        <v>60628959.79</v>
+        <v>-0</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -17516,7 +17591,7 @@
         <v>33122800.6</v>
       </c>
       <c r="F4" t="n">
-        <v>46181445.83</v>
+        <v>-0</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -17546,7 +17621,7 @@
         <v>41417</v>
       </c>
       <c r="F5" t="n">
-        <v>46477</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -17557,6 +17632,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -17564,7 +17640,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>370</v>
+        <v>385</v>
       </c>
     </row>
     <row r="8">
@@ -17574,7 +17650,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -17584,7 +17660,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -17617,6 +17693,7 @@
         <v>398</v>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -17675,6 +17752,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -17683,8 +17761,50 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>indisponible : décisions à prendre</t>
-        </is>
+          <t>possible (case à cocher par Baptiste)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Prise en compte des décisions</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Décisions « Oui »</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Décisions « Non »</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Décisions manquantes</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>